<commit_message>
chore(narjiss): médias des plans (découpes jawhara + plans andalusia) et évolutions en cours du site
- médias : plans immeubles jawhara + 70 vignettes par lot (jawhara/plans/lots),
  plans andalusia, plan-masse ; plans travaillés jawhara/floorplan.
- données : grilles de lots jawhara/andalusia (data/lots), data/projects.json.
- back-office & outils en cours : admin/lots*, api/lots-*, api/xlsx-lib.php,
  sql (migrer, etat, 003/…), tools de génération de lots.
- pages et menu partagé mis à jour ; deploy.sh ; .gitignore (exclut
  data/videos, data/backups, outputs).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/lots/narjiss-lots-jawhara-demo.xlsx
+++ b/data/lots/narjiss-lots-jawhara-demo.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Listes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lots'!$A$1:$T$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Lots'!$A$1:$W$91</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -816,7 +816,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T91"/>
+  <dimension ref="A1:W91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -838,7 +838,9 @@
     <col width="13" customWidth="1" min="17" max="17"/>
     <col width="16" customWidth="1" min="18" max="18"/>
     <col width="30" customWidth="1" min="19" max="19"/>
-    <col width="40" customWidth="1" min="20" max="20"/>
+    <col width="34" customWidth="1" min="20" max="20"/>
+    <col width="34" customWidth="1" min="21" max="21"/>
+    <col width="34" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -937,7 +939,22 @@
           <t>plan_fichier</t>
         </is>
       </c>
-      <c r="T1" s="6" t="inlineStr">
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>plan_architecte</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>plan_visuel</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>visite_360</t>
+        </is>
+      </c>
+      <c r="W1" s="6" t="inlineStr">
         <is>
           <t>notes</t>
         </is>
@@ -1019,7 +1036,22 @@
       </c>
       <c r="R2" s="8" t="inlineStr"/>
       <c r="S2" s="15" t="inlineStr"/>
-      <c r="T2" s="15" t="inlineStr">
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W2" s="15" t="inlineStr">
         <is>
           <t>Local commercial avec vitrine sur la voie principale</t>
         </is>
@@ -1105,7 +1137,22 @@
         </is>
       </c>
       <c r="S3" s="15" t="inlineStr"/>
-      <c r="T3" s="15" t="inlineStr">
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W3" s="15" t="inlineStr">
         <is>
           <t>Local commercial avec vitrine sur la voie principale</t>
         </is>
@@ -1187,7 +1234,22 @@
       </c>
       <c r="R4" s="8" t="inlineStr"/>
       <c r="S4" s="15" t="inlineStr"/>
-      <c r="T4" s="15" t="inlineStr">
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W4" s="15" t="inlineStr">
         <is>
           <t>Plateau de bureau modulable, entree independante</t>
         </is>
@@ -1269,7 +1331,22 @@
       </c>
       <c r="R5" s="8" t="inlineStr"/>
       <c r="S5" s="15" t="inlineStr"/>
-      <c r="T5" s="15" t="inlineStr">
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W5" s="15" t="inlineStr">
         <is>
           <t>Acces direct au jardin interieur, ideal pour une famille</t>
         </is>
@@ -1351,7 +1428,22 @@
       </c>
       <c r="R6" s="8" t="inlineStr"/>
       <c r="S6" s="15" t="inlineStr"/>
-      <c r="T6" s="15" t="inlineStr">
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W6" s="15" t="inlineStr">
         <is>
           <t>Acces direct au jardin interieur, ideal pour une famille</t>
         </is>
@@ -1433,7 +1525,22 @@
       </c>
       <c r="R7" s="8" t="inlineStr"/>
       <c r="S7" s="15" t="inlineStr"/>
-      <c r="T7" s="15" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W7" s="15" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -1511,7 +1618,22 @@
       </c>
       <c r="R8" s="8" t="inlineStr"/>
       <c r="S8" s="15" t="inlineStr"/>
-      <c r="T8" s="15" t="inlineStr"/>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W8" s="15" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
@@ -1589,7 +1711,22 @@
       </c>
       <c r="R9" s="8" t="inlineStr"/>
       <c r="S9" s="15" t="inlineStr"/>
-      <c r="T9" s="15" t="inlineStr"/>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W9" s="15" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -1667,7 +1804,22 @@
       </c>
       <c r="R10" s="8" t="inlineStr"/>
       <c r="S10" s="15" t="inlineStr"/>
-      <c r="T10" s="15" t="inlineStr"/>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W10" s="15" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -1745,7 +1897,22 @@
       </c>
       <c r="R11" s="8" t="inlineStr"/>
       <c r="S11" s="15" t="inlineStr"/>
-      <c r="T11" s="15" t="inlineStr"/>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W11" s="15" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -1823,7 +1990,22 @@
       </c>
       <c r="R12" s="8" t="inlineStr"/>
       <c r="S12" s="15" t="inlineStr"/>
-      <c r="T12" s="15" t="inlineStr">
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W12" s="15" t="inlineStr">
         <is>
           <t>Traversant : lumiere du matin et du soir</t>
         </is>
@@ -1905,7 +2087,22 @@
       </c>
       <c r="R13" s="8" t="inlineStr"/>
       <c r="S13" s="15" t="inlineStr"/>
-      <c r="T13" s="15" t="inlineStr">
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W13" s="15" t="inlineStr">
         <is>
           <t>Appartement d'angle, deux facades</t>
         </is>
@@ -1987,7 +2184,22 @@
       </c>
       <c r="R14" s="8" t="inlineStr"/>
       <c r="S14" s="15" t="inlineStr"/>
-      <c r="T14" s="15" t="inlineStr"/>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W14" s="15" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -2065,7 +2277,22 @@
       </c>
       <c r="R15" s="8" t="inlineStr"/>
       <c r="S15" s="15" t="inlineStr"/>
-      <c r="T15" s="15" t="inlineStr"/>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W15" s="15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -2143,7 +2370,22 @@
       </c>
       <c r="R16" s="8" t="inlineStr"/>
       <c r="S16" s="15" t="inlineStr"/>
-      <c r="T16" s="15" t="inlineStr">
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W16" s="15" t="inlineStr">
         <is>
           <t>Logement temoin, non commercialise</t>
         </is>
@@ -2225,7 +2467,22 @@
       </c>
       <c r="R17" s="8" t="inlineStr"/>
       <c r="S17" s="15" t="inlineStr"/>
-      <c r="T17" s="15" t="inlineStr"/>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W17" s="15" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -2303,7 +2560,22 @@
       </c>
       <c r="R18" s="8" t="inlineStr"/>
       <c r="S18" s="15" t="inlineStr"/>
-      <c r="T18" s="15" t="inlineStr">
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W18" s="15" t="inlineStr">
         <is>
           <t>Traversant : lumiere du matin et du soir</t>
         </is>
@@ -2385,7 +2657,22 @@
       </c>
       <c r="R19" s="8" t="inlineStr"/>
       <c r="S19" s="15" t="inlineStr"/>
-      <c r="T19" s="15" t="inlineStr">
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W19" s="15" t="inlineStr">
         <is>
           <t>Appartement d'angle, deux facades</t>
         </is>
@@ -2467,7 +2754,22 @@
       </c>
       <c r="R20" s="8" t="inlineStr"/>
       <c r="S20" s="15" t="inlineStr"/>
-      <c r="T20" s="15" t="inlineStr"/>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W20" s="15" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
@@ -2545,7 +2847,22 @@
       </c>
       <c r="R21" s="8" t="inlineStr"/>
       <c r="S21" s="15" t="inlineStr"/>
-      <c r="T21" s="15" t="inlineStr"/>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W21" s="15" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
@@ -2623,7 +2940,22 @@
       </c>
       <c r="R22" s="8" t="inlineStr"/>
       <c r="S22" s="15" t="inlineStr"/>
-      <c r="T22" s="15" t="inlineStr"/>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W22" s="15" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
@@ -2701,7 +3033,22 @@
       </c>
       <c r="R23" s="8" t="inlineStr"/>
       <c r="S23" s="15" t="inlineStr"/>
-      <c r="T23" s="15" t="inlineStr"/>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W23" s="15" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
@@ -2779,7 +3126,22 @@
       </c>
       <c r="R24" s="8" t="inlineStr"/>
       <c r="S24" s="15" t="inlineStr"/>
-      <c r="T24" s="15" t="inlineStr">
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W24" s="15" t="inlineStr">
         <is>
           <t>Traversant : lumiere du matin et du soir</t>
         </is>
@@ -2861,7 +3223,22 @@
       </c>
       <c r="R25" s="8" t="inlineStr"/>
       <c r="S25" s="15" t="inlineStr"/>
-      <c r="T25" s="15" t="inlineStr">
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W25" s="15" t="inlineStr">
         <is>
           <t>Appartement d'angle, deux facades</t>
         </is>
@@ -2943,7 +3320,22 @@
       </c>
       <c r="R26" s="8" t="inlineStr"/>
       <c r="S26" s="15" t="inlineStr"/>
-      <c r="T26" s="15" t="inlineStr">
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W26" s="15" t="inlineStr">
         <is>
           <t>Duplex avec terrasse privative, vue degagee sur l'Atlas</t>
         </is>
@@ -3025,7 +3417,22 @@
       </c>
       <c r="R27" s="8" t="inlineStr"/>
       <c r="S27" s="15" t="inlineStr"/>
-      <c r="T27" s="15" t="inlineStr">
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W27" s="15" t="inlineStr">
         <is>
           <t>Dernier etage, terrasse privative</t>
         </is>
@@ -3107,7 +3514,22 @@
       </c>
       <c r="R28" s="8" t="inlineStr"/>
       <c r="S28" s="15" t="inlineStr"/>
-      <c r="T28" s="15" t="inlineStr">
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W28" s="15" t="inlineStr">
         <is>
           <t>Dernier etage, terrasse privative</t>
         </is>
@@ -3189,7 +3611,22 @@
       </c>
       <c r="R29" s="8" t="inlineStr"/>
       <c r="S29" s="15" t="inlineStr"/>
-      <c r="T29" s="15" t="inlineStr">
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W29" s="15" t="inlineStr">
         <is>
           <t>Dernier etage, terrasse privative</t>
         </is>
@@ -3271,7 +3708,22 @@
       </c>
       <c r="R30" s="8" t="inlineStr"/>
       <c r="S30" s="15" t="inlineStr"/>
-      <c r="T30" s="15" t="inlineStr">
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W30" s="15" t="inlineStr">
         <is>
           <t>Duplex avec terrasse privative, vue degagee sur l'Atlas</t>
         </is>
@@ -3357,7 +3809,22 @@
         </is>
       </c>
       <c r="S31" s="15" t="inlineStr"/>
-      <c r="T31" s="15" t="inlineStr">
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W31" s="15" t="inlineStr">
         <is>
           <t>Dernier etage, terrasse privative</t>
         </is>
@@ -3439,7 +3906,22 @@
       </c>
       <c r="R32" s="8" t="inlineStr"/>
       <c r="S32" s="15" t="inlineStr"/>
-      <c r="T32" s="15" t="inlineStr">
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W32" s="15" t="inlineStr">
         <is>
           <t>Local commercial avec vitrine sur la voie principale</t>
         </is>
@@ -3521,7 +4003,22 @@
       </c>
       <c r="R33" s="8" t="inlineStr"/>
       <c r="S33" s="15" t="inlineStr"/>
-      <c r="T33" s="15" t="inlineStr">
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W33" s="15" t="inlineStr">
         <is>
           <t>Local commercial avec vitrine sur la voie principale</t>
         </is>
@@ -3603,7 +4100,22 @@
       </c>
       <c r="R34" s="8" t="inlineStr"/>
       <c r="S34" s="15" t="inlineStr"/>
-      <c r="T34" s="15" t="inlineStr">
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W34" s="15" t="inlineStr">
         <is>
           <t>Plateau de bureau modulable, entree independante</t>
         </is>
@@ -3685,7 +4197,22 @@
       </c>
       <c r="R35" s="8" t="inlineStr"/>
       <c r="S35" s="15" t="inlineStr"/>
-      <c r="T35" s="15" t="inlineStr">
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W35" s="15" t="inlineStr">
         <is>
           <t>Acces direct au jardin interieur, ideal pour une famille</t>
         </is>
@@ -3767,7 +4294,22 @@
       </c>
       <c r="R36" s="8" t="inlineStr"/>
       <c r="S36" s="15" t="inlineStr"/>
-      <c r="T36" s="15" t="inlineStr">
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W36" s="15" t="inlineStr">
         <is>
           <t>Acces direct au jardin interieur, ideal pour une famille</t>
         </is>
@@ -3849,7 +4391,22 @@
       </c>
       <c r="R37" s="8" t="inlineStr"/>
       <c r="S37" s="15" t="inlineStr"/>
-      <c r="T37" s="15" t="inlineStr"/>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W37" s="15" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="8" t="inlineStr">
@@ -3927,7 +4484,22 @@
       </c>
       <c r="R38" s="8" t="inlineStr"/>
       <c r="S38" s="15" t="inlineStr"/>
-      <c r="T38" s="15" t="inlineStr"/>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W38" s="15" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
@@ -4009,7 +4581,22 @@
         </is>
       </c>
       <c r="S39" s="15" t="inlineStr"/>
-      <c r="T39" s="15" t="inlineStr"/>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W39" s="15" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
@@ -4087,7 +4674,22 @@
       </c>
       <c r="R40" s="8" t="inlineStr"/>
       <c r="S40" s="15" t="inlineStr"/>
-      <c r="T40" s="15" t="inlineStr"/>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W40" s="15" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
@@ -4165,7 +4767,22 @@
       </c>
       <c r="R41" s="8" t="inlineStr"/>
       <c r="S41" s="15" t="inlineStr"/>
-      <c r="T41" s="15" t="inlineStr"/>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W41" s="15" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
@@ -4243,7 +4860,22 @@
       </c>
       <c r="R42" s="8" t="inlineStr"/>
       <c r="S42" s="15" t="inlineStr"/>
-      <c r="T42" s="15" t="inlineStr">
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W42" s="15" t="inlineStr">
         <is>
           <t>Traversant : lumiere du matin et du soir</t>
         </is>
@@ -4325,7 +4957,22 @@
       </c>
       <c r="R43" s="8" t="inlineStr"/>
       <c r="S43" s="15" t="inlineStr"/>
-      <c r="T43" s="15" t="inlineStr">
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W43" s="15" t="inlineStr">
         <is>
           <t>Appartement d'angle, deux facades</t>
         </is>
@@ -4407,7 +5054,22 @@
       </c>
       <c r="R44" s="8" t="inlineStr"/>
       <c r="S44" s="15" t="inlineStr"/>
-      <c r="T44" s="15" t="inlineStr"/>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W44" s="15" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
@@ -4485,7 +5147,22 @@
       </c>
       <c r="R45" s="8" t="inlineStr"/>
       <c r="S45" s="15" t="inlineStr"/>
-      <c r="T45" s="15" t="inlineStr"/>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W45" s="15" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
@@ -4563,7 +5240,22 @@
       </c>
       <c r="R46" s="8" t="inlineStr"/>
       <c r="S46" s="15" t="inlineStr"/>
-      <c r="T46" s="15" t="inlineStr">
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W46" s="15" t="inlineStr">
         <is>
           <t>Logement temoin, non commercialise</t>
         </is>
@@ -4645,7 +5337,22 @@
       </c>
       <c r="R47" s="8" t="inlineStr"/>
       <c r="S47" s="15" t="inlineStr"/>
-      <c r="T47" s="15" t="inlineStr"/>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W47" s="15" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
@@ -4723,7 +5430,22 @@
       </c>
       <c r="R48" s="8" t="inlineStr"/>
       <c r="S48" s="15" t="inlineStr"/>
-      <c r="T48" s="15" t="inlineStr">
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W48" s="15" t="inlineStr">
         <is>
           <t>Traversant : lumiere du matin et du soir</t>
         </is>
@@ -4805,7 +5527,22 @@
       </c>
       <c r="R49" s="8" t="inlineStr"/>
       <c r="S49" s="15" t="inlineStr"/>
-      <c r="T49" s="15" t="inlineStr">
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W49" s="15" t="inlineStr">
         <is>
           <t>Appartement d'angle, deux facades</t>
         </is>
@@ -4887,7 +5624,22 @@
       </c>
       <c r="R50" s="8" t="inlineStr"/>
       <c r="S50" s="15" t="inlineStr"/>
-      <c r="T50" s="15" t="inlineStr"/>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W50" s="15" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
@@ -4965,7 +5717,22 @@
       </c>
       <c r="R51" s="8" t="inlineStr"/>
       <c r="S51" s="15" t="inlineStr"/>
-      <c r="T51" s="15" t="inlineStr"/>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W51" s="15" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
@@ -5047,7 +5814,22 @@
         </is>
       </c>
       <c r="S52" s="15" t="inlineStr"/>
-      <c r="T52" s="15" t="inlineStr"/>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W52" s="15" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
@@ -5125,7 +5907,22 @@
       </c>
       <c r="R53" s="8" t="inlineStr"/>
       <c r="S53" s="15" t="inlineStr"/>
-      <c r="T53" s="15" t="inlineStr"/>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W53" s="15" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
@@ -5203,7 +6000,22 @@
       </c>
       <c r="R54" s="8" t="inlineStr"/>
       <c r="S54" s="15" t="inlineStr"/>
-      <c r="T54" s="15" t="inlineStr">
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W54" s="15" t="inlineStr">
         <is>
           <t>Traversant : lumiere du matin et du soir</t>
         </is>
@@ -5285,7 +6097,22 @@
       </c>
       <c r="R55" s="8" t="inlineStr"/>
       <c r="S55" s="15" t="inlineStr"/>
-      <c r="T55" s="15" t="inlineStr">
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W55" s="15" t="inlineStr">
         <is>
           <t>Appartement d'angle, deux facades</t>
         </is>
@@ -5367,7 +6194,22 @@
       </c>
       <c r="R56" s="8" t="inlineStr"/>
       <c r="S56" s="15" t="inlineStr"/>
-      <c r="T56" s="15" t="inlineStr">
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W56" s="15" t="inlineStr">
         <is>
           <t>Duplex avec terrasse privative, vue degagee sur l'Atlas</t>
         </is>
@@ -5449,7 +6291,22 @@
       </c>
       <c r="R57" s="8" t="inlineStr"/>
       <c r="S57" s="15" t="inlineStr"/>
-      <c r="T57" s="15" t="inlineStr">
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W57" s="15" t="inlineStr">
         <is>
           <t>Dernier etage, terrasse privative</t>
         </is>
@@ -5535,7 +6392,22 @@
         </is>
       </c>
       <c r="S58" s="15" t="inlineStr"/>
-      <c r="T58" s="15" t="inlineStr">
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W58" s="15" t="inlineStr">
         <is>
           <t>Dernier etage, terrasse privative</t>
         </is>
@@ -5617,7 +6489,22 @@
       </c>
       <c r="R59" s="8" t="inlineStr"/>
       <c r="S59" s="15" t="inlineStr"/>
-      <c r="T59" s="15" t="inlineStr">
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W59" s="15" t="inlineStr">
         <is>
           <t>Dernier etage, terrasse privative</t>
         </is>
@@ -5699,7 +6586,22 @@
       </c>
       <c r="R60" s="8" t="inlineStr"/>
       <c r="S60" s="15" t="inlineStr"/>
-      <c r="T60" s="15" t="inlineStr">
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W60" s="15" t="inlineStr">
         <is>
           <t>Duplex avec terrasse privative, vue degagee sur l'Atlas</t>
         </is>
@@ -5781,7 +6683,22 @@
       </c>
       <c r="R61" s="8" t="inlineStr"/>
       <c r="S61" s="15" t="inlineStr"/>
-      <c r="T61" s="15" t="inlineStr">
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W61" s="15" t="inlineStr">
         <is>
           <t>Dernier etage, terrasse privative</t>
         </is>
@@ -5863,7 +6780,22 @@
       </c>
       <c r="R62" s="8" t="inlineStr"/>
       <c r="S62" s="15" t="inlineStr"/>
-      <c r="T62" s="15" t="inlineStr">
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W62" s="15" t="inlineStr">
         <is>
           <t>Local commercial avec vitrine sur la voie principale</t>
         </is>
@@ -5945,7 +6877,22 @@
       </c>
       <c r="R63" s="8" t="inlineStr"/>
       <c r="S63" s="15" t="inlineStr"/>
-      <c r="T63" s="15" t="inlineStr">
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W63" s="15" t="inlineStr">
         <is>
           <t>Local commercial avec vitrine sur la voie principale</t>
         </is>
@@ -6027,7 +6974,22 @@
       </c>
       <c r="R64" s="8" t="inlineStr"/>
       <c r="S64" s="15" t="inlineStr"/>
-      <c r="T64" s="15" t="inlineStr">
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W64" s="15" t="inlineStr">
         <is>
           <t>Plateau de bureau modulable, entree independante</t>
         </is>
@@ -6109,7 +7071,22 @@
       </c>
       <c r="R65" s="8" t="inlineStr"/>
       <c r="S65" s="15" t="inlineStr"/>
-      <c r="T65" s="15" t="inlineStr">
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W65" s="15" t="inlineStr">
         <is>
           <t>Acces direct au jardin interieur, ideal pour une famille</t>
         </is>
@@ -6195,7 +7172,22 @@
         </is>
       </c>
       <c r="S66" s="15" t="inlineStr"/>
-      <c r="T66" s="15" t="inlineStr">
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W66" s="15" t="inlineStr">
         <is>
           <t>Acces direct au jardin interieur, ideal pour une famille</t>
         </is>
@@ -6277,7 +7269,22 @@
       </c>
       <c r="R67" s="8" t="inlineStr"/>
       <c r="S67" s="15" t="inlineStr"/>
-      <c r="T67" s="15" t="inlineStr"/>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W67" s="15" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
@@ -6355,7 +7362,22 @@
       </c>
       <c r="R68" s="8" t="inlineStr"/>
       <c r="S68" s="15" t="inlineStr"/>
-      <c r="T68" s="15" t="inlineStr"/>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W68" s="15" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
@@ -6433,7 +7455,22 @@
       </c>
       <c r="R69" s="8" t="inlineStr"/>
       <c r="S69" s="15" t="inlineStr"/>
-      <c r="T69" s="15" t="inlineStr"/>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W69" s="15" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
@@ -6511,7 +7548,22 @@
       </c>
       <c r="R70" s="8" t="inlineStr"/>
       <c r="S70" s="15" t="inlineStr"/>
-      <c r="T70" s="15" t="inlineStr"/>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W70" s="15" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="8" t="inlineStr">
@@ -6589,7 +7641,22 @@
       </c>
       <c r="R71" s="8" t="inlineStr"/>
       <c r="S71" s="15" t="inlineStr"/>
-      <c r="T71" s="15" t="inlineStr"/>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W71" s="15" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="8" t="inlineStr">
@@ -6667,7 +7734,22 @@
       </c>
       <c r="R72" s="8" t="inlineStr"/>
       <c r="S72" s="15" t="inlineStr"/>
-      <c r="T72" s="15" t="inlineStr">
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W72" s="15" t="inlineStr">
         <is>
           <t>Traversant : lumiere du matin et du soir</t>
         </is>
@@ -6749,7 +7831,22 @@
       </c>
       <c r="R73" s="8" t="inlineStr"/>
       <c r="S73" s="15" t="inlineStr"/>
-      <c r="T73" s="15" t="inlineStr">
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W73" s="15" t="inlineStr">
         <is>
           <t>Appartement d'angle, deux facades</t>
         </is>
@@ -6831,7 +7928,22 @@
       </c>
       <c r="R74" s="8" t="inlineStr"/>
       <c r="S74" s="15" t="inlineStr"/>
-      <c r="T74" s="15" t="inlineStr"/>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W74" s="15" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="8" t="inlineStr">
@@ -6909,7 +8021,22 @@
       </c>
       <c r="R75" s="8" t="inlineStr"/>
       <c r="S75" s="15" t="inlineStr"/>
-      <c r="T75" s="15" t="inlineStr"/>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W75" s="15" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="8" t="inlineStr">
@@ -6987,7 +8114,22 @@
       </c>
       <c r="R76" s="8" t="inlineStr"/>
       <c r="S76" s="15" t="inlineStr"/>
-      <c r="T76" s="15" t="inlineStr">
+      <c r="T76" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V76" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W76" s="15" t="inlineStr">
         <is>
           <t>Logement temoin, non commercialise</t>
         </is>
@@ -7069,7 +8211,22 @@
       </c>
       <c r="R77" s="8" t="inlineStr"/>
       <c r="S77" s="15" t="inlineStr"/>
-      <c r="T77" s="15" t="inlineStr"/>
+      <c r="T77" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W77" s="15" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="8" t="inlineStr">
@@ -7147,7 +8304,22 @@
       </c>
       <c r="R78" s="8" t="inlineStr"/>
       <c r="S78" s="15" t="inlineStr"/>
-      <c r="T78" s="15" t="inlineStr">
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V78" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W78" s="15" t="inlineStr">
         <is>
           <t>Traversant : lumiere du matin et du soir</t>
         </is>
@@ -7229,7 +8401,22 @@
       </c>
       <c r="R79" s="8" t="inlineStr"/>
       <c r="S79" s="15" t="inlineStr"/>
-      <c r="T79" s="15" t="inlineStr">
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V79" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W79" s="15" t="inlineStr">
         <is>
           <t>Appartement d'angle, deux facades</t>
         </is>
@@ -7311,7 +8498,22 @@
       </c>
       <c r="R80" s="8" t="inlineStr"/>
       <c r="S80" s="15" t="inlineStr"/>
-      <c r="T80" s="15" t="inlineStr"/>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V80" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W80" s="15" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="8" t="inlineStr">
@@ -7389,7 +8591,22 @@
       </c>
       <c r="R81" s="8" t="inlineStr"/>
       <c r="S81" s="15" t="inlineStr"/>
-      <c r="T81" s="15" t="inlineStr"/>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V81" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W81" s="15" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="8" t="inlineStr">
@@ -7467,7 +8684,22 @@
       </c>
       <c r="R82" s="8" t="inlineStr"/>
       <c r="S82" s="15" t="inlineStr"/>
-      <c r="T82" s="15" t="inlineStr"/>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V82" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W82" s="15" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="8" t="inlineStr">
@@ -7545,7 +8777,22 @@
       </c>
       <c r="R83" s="8" t="inlineStr"/>
       <c r="S83" s="15" t="inlineStr"/>
-      <c r="T83" s="15" t="inlineStr"/>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V83" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W83" s="15" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="8" t="inlineStr">
@@ -7623,7 +8870,22 @@
       </c>
       <c r="R84" s="8" t="inlineStr"/>
       <c r="S84" s="15" t="inlineStr"/>
-      <c r="T84" s="15" t="inlineStr">
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V84" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W84" s="15" t="inlineStr">
         <is>
           <t>Traversant : lumiere du matin et du soir</t>
         </is>
@@ -7705,7 +8967,22 @@
       </c>
       <c r="R85" s="8" t="inlineStr"/>
       <c r="S85" s="15" t="inlineStr"/>
-      <c r="T85" s="15" t="inlineStr">
+      <c r="T85" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U85" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V85" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W85" s="15" t="inlineStr">
         <is>
           <t>Appartement d'angle, deux facades</t>
         </is>
@@ -7787,7 +9064,22 @@
       </c>
       <c r="R86" s="8" t="inlineStr"/>
       <c r="S86" s="15" t="inlineStr"/>
-      <c r="T86" s="15" t="inlineStr">
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U86" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V86" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W86" s="15" t="inlineStr">
         <is>
           <t>Duplex avec terrasse privative, vue degagee sur l'Atlas</t>
         </is>
@@ -7869,7 +9161,22 @@
       </c>
       <c r="R87" s="8" t="inlineStr"/>
       <c r="S87" s="15" t="inlineStr"/>
-      <c r="T87" s="15" t="inlineStr">
+      <c r="T87" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U87" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V87" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W87" s="15" t="inlineStr">
         <is>
           <t>Dernier etage, terrasse privative</t>
         </is>
@@ -7951,7 +9258,22 @@
       </c>
       <c r="R88" s="8" t="inlineStr"/>
       <c r="S88" s="15" t="inlineStr"/>
-      <c r="T88" s="15" t="inlineStr">
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V88" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W88" s="15" t="inlineStr">
         <is>
           <t>Dernier etage, terrasse privative</t>
         </is>
@@ -8033,7 +9355,22 @@
       </c>
       <c r="R89" s="8" t="inlineStr"/>
       <c r="S89" s="15" t="inlineStr"/>
-      <c r="T89" s="15" t="inlineStr">
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U89" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V89" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W89" s="15" t="inlineStr">
         <is>
           <t>Dernier etage, terrasse privative</t>
         </is>
@@ -8115,7 +9452,22 @@
       </c>
       <c r="R90" s="8" t="inlineStr"/>
       <c r="S90" s="15" t="inlineStr"/>
-      <c r="T90" s="15" t="inlineStr">
+      <c r="T90" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U90" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V90" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W90" s="15" t="inlineStr">
         <is>
           <t>Duplex avec terrasse privative, vue degagee sur l'Atlas</t>
         </is>
@@ -8197,14 +9549,29 @@
       </c>
       <c r="R91" s="8" t="inlineStr"/>
       <c r="S91" s="15" t="inlineStr"/>
-      <c r="T91" s="15" t="inlineStr">
+      <c r="T91" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-architecte.png</t>
+        </is>
+      </c>
+      <c r="U91" t="inlineStr">
+        <is>
+          <t>jawhara/floorplan/plan-visuel.jpg</t>
+        </is>
+      </c>
+      <c r="V91" t="inlineStr">
+        <is>
+          <t>jawhara/Tour-FloorPlan/index.htm</t>
+        </is>
+      </c>
+      <c r="W91" s="15" t="inlineStr">
         <is>
           <t>Dernier etage, terrasse privative</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T91"/>
+  <autoFilter ref="A1:W91"/>
   <dataValidations count="8">
     <dataValidation sqref="E2:E490" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Saisie invalide" error="Valeur non autorisee. Choisir dans la liste." type="list">
       <formula1>"Studio,F2,F3,F4,F5,Duplex,Bureau,Commerce"</formula1>

</xml_diff>

<commit_message>
chore(lots): aligner les classeurs Excel sur la palette des statuts
La grille du bureau de vente affichait encore l'ancien code couleur (vert
pastel, jaune, orange, gris) : elle contredisait desormais le plan que voit le
client. Les aplats des onglets Lots et Synthese passent aux teintes du site,
avec l'encre exacte de statuts-lots.css.

Une mise en forme conditionnelle est en plus posee sur la colonne statut
(Q2:Q1000) des deux classeurs : une ligne saisie plus tard se colore seule. Le
modele vierge n'avait aucune couleur — le bureau de vente les posait a la main,
donc au petit bonheur.

L'onglet Notice est laisse tel quel : il surligne ses questions au client avec
le meme jaune que l'ancien << optionne >>, sans vouloir dire un statut.

tools/recolorer-lots-xlsx.py rejoue l'operation sur une autre grille.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/lots/narjiss-lots-jawhara-demo.xlsx
+++ b/data/lots/narjiss-lots-jawhara-demo.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,8 +77,63 @@
       <color rgb="00808080"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F6F55"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="009E6300"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="005A6272"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001C5FA8"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00B02A2A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001F6F55"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="009E6300"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="001C5FA8"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="005A6272"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00B02A2A"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -128,6 +183,36 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E4F1EA"/>
+        <bgColor rgb="00E4F1EA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FBEEDA"/>
+        <bgColor rgb="00FBEEDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00ECEEF1"/>
+        <bgColor rgb="00ECEEF1"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E3EDF9"/>
+        <bgColor rgb="00E3EDF9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7DEDE"/>
+        <bgColor rgb="00F7DEDE"/>
       </patternFill>
     </fill>
   </fills>
@@ -190,7 +275,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" indent="1"/>
@@ -277,10 +362,97 @@
       <alignment horizontal="right" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="5">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="001F6F55"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="00E4F1EA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="009E6300"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="00FBEEDA"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="001C5FA8"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="00E3EDF9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="005A6272"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="00ECEEF1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="00B02A2A"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="00F7DEDE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -1029,7 +1201,7 @@
         <f>IFERROR(O2/F2,"")</f>
         <v/>
       </c>
-      <c r="Q2" s="14" t="inlineStr">
+      <c r="Q2" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -1126,7 +1298,7 @@
         <f>IFERROR(O3/F3,"")</f>
         <v/>
       </c>
-      <c r="Q3" s="16" t="inlineStr">
+      <c r="Q3" s="35" t="inlineStr">
         <is>
           <t>Optionne</t>
         </is>
@@ -1227,7 +1399,7 @@
         <f>IFERROR(O4/F4,"")</f>
         <v/>
       </c>
-      <c r="Q4" s="17" t="inlineStr">
+      <c r="Q4" s="36" t="inlineStr">
         <is>
           <t>Vendu</t>
         </is>
@@ -1324,7 +1496,7 @@
         <f>IFERROR(O5/F5,"")</f>
         <v/>
       </c>
-      <c r="Q5" s="14" t="inlineStr">
+      <c r="Q5" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -1421,7 +1593,7 @@
         <f>IFERROR(O6/F6,"")</f>
         <v/>
       </c>
-      <c r="Q6" s="18" t="inlineStr">
+      <c r="Q6" s="37" t="inlineStr">
         <is>
           <t>Reserve</t>
         </is>
@@ -1518,7 +1690,7 @@
         <f>IFERROR(O7/F7,"")</f>
         <v/>
       </c>
-      <c r="Q7" s="17" t="inlineStr">
+      <c r="Q7" s="36" t="inlineStr">
         <is>
           <t>Vendu</t>
         </is>
@@ -1611,7 +1783,7 @@
         <f>IFERROR(O8/F8,"")</f>
         <v/>
       </c>
-      <c r="Q8" s="17" t="inlineStr">
+      <c r="Q8" s="36" t="inlineStr">
         <is>
           <t>Vendu</t>
         </is>
@@ -1704,7 +1876,7 @@
         <f>IFERROR(O9/F9,"")</f>
         <v/>
       </c>
-      <c r="Q9" s="14" t="inlineStr">
+      <c r="Q9" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -1797,7 +1969,7 @@
         <f>IFERROR(O10/F10,"")</f>
         <v/>
       </c>
-      <c r="Q10" s="17" t="inlineStr">
+      <c r="Q10" s="36" t="inlineStr">
         <is>
           <t>Vendu</t>
         </is>
@@ -1890,7 +2062,7 @@
         <f>IFERROR(O11/F11,"")</f>
         <v/>
       </c>
-      <c r="Q11" s="17" t="inlineStr">
+      <c r="Q11" s="36" t="inlineStr">
         <is>
           <t>Vendu</t>
         </is>
@@ -1983,7 +2155,7 @@
         <f>IFERROR(O12/F12,"")</f>
         <v/>
       </c>
-      <c r="Q12" s="18" t="inlineStr">
+      <c r="Q12" s="37" t="inlineStr">
         <is>
           <t>Reserve</t>
         </is>
@@ -2080,7 +2252,7 @@
         <f>IFERROR(O13/F13,"")</f>
         <v/>
       </c>
-      <c r="Q13" s="17" t="inlineStr">
+      <c r="Q13" s="36" t="inlineStr">
         <is>
           <t>Vendu</t>
         </is>
@@ -2177,7 +2349,7 @@
         <f>IFERROR(O14/F14,"")</f>
         <v/>
       </c>
-      <c r="Q14" s="18" t="inlineStr">
+      <c r="Q14" s="37" t="inlineStr">
         <is>
           <t>Reserve</t>
         </is>
@@ -2270,7 +2442,7 @@
         <f>IFERROR(O15/F15,"")</f>
         <v/>
       </c>
-      <c r="Q15" s="14" t="inlineStr">
+      <c r="Q15" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -2363,7 +2535,7 @@
         <f>IFERROR(O16/F16,"")</f>
         <v/>
       </c>
-      <c r="Q16" s="19" t="inlineStr">
+      <c r="Q16" s="38" t="inlineStr">
         <is>
           <t>Bloque</t>
         </is>
@@ -2460,7 +2632,7 @@
         <f>IFERROR(O17/F17,"")</f>
         <v/>
       </c>
-      <c r="Q17" s="18" t="inlineStr">
+      <c r="Q17" s="37" t="inlineStr">
         <is>
           <t>Reserve</t>
         </is>
@@ -2553,7 +2725,7 @@
         <f>IFERROR(O18/F18,"")</f>
         <v/>
       </c>
-      <c r="Q18" s="14" t="inlineStr">
+      <c r="Q18" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -2650,7 +2822,7 @@
         <f>IFERROR(O19/F19,"")</f>
         <v/>
       </c>
-      <c r="Q19" s="14" t="inlineStr">
+      <c r="Q19" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -2747,7 +2919,7 @@
         <f>IFERROR(O20/F20,"")</f>
         <v/>
       </c>
-      <c r="Q20" s="14" t="inlineStr">
+      <c r="Q20" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -2840,7 +3012,7 @@
         <f>IFERROR(O21/F21,"")</f>
         <v/>
       </c>
-      <c r="Q21" s="17" t="inlineStr">
+      <c r="Q21" s="36" t="inlineStr">
         <is>
           <t>Vendu</t>
         </is>
@@ -2933,7 +3105,7 @@
         <f>IFERROR(O22/F22,"")</f>
         <v/>
       </c>
-      <c r="Q22" s="14" t="inlineStr">
+      <c r="Q22" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -3026,7 +3198,7 @@
         <f>IFERROR(O23/F23,"")</f>
         <v/>
       </c>
-      <c r="Q23" s="17" t="inlineStr">
+      <c r="Q23" s="36" t="inlineStr">
         <is>
           <t>Vendu</t>
         </is>
@@ -3119,7 +3291,7 @@
         <f>IFERROR(O24/F24,"")</f>
         <v/>
       </c>
-      <c r="Q24" s="17" t="inlineStr">
+      <c r="Q24" s="36" t="inlineStr">
         <is>
           <t>Vendu</t>
         </is>
@@ -3216,7 +3388,7 @@
         <f>IFERROR(O25/F25,"")</f>
         <v/>
       </c>
-      <c r="Q25" s="14" t="inlineStr">
+      <c r="Q25" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -3313,7 +3485,7 @@
         <f>IFERROR(O26/F26,"")</f>
         <v/>
       </c>
-      <c r="Q26" s="17" t="inlineStr">
+      <c r="Q26" s="36" t="inlineStr">
         <is>
           <t>Vendu</t>
         </is>
@@ -3410,7 +3582,7 @@
         <f>IFERROR(O27/F27,"")</f>
         <v/>
       </c>
-      <c r="Q27" s="18" t="inlineStr">
+      <c r="Q27" s="37" t="inlineStr">
         <is>
           <t>Reserve</t>
         </is>
@@ -3507,7 +3679,7 @@
         <f>IFERROR(O28/F28,"")</f>
         <v/>
       </c>
-      <c r="Q28" s="18" t="inlineStr">
+      <c r="Q28" s="37" t="inlineStr">
         <is>
           <t>Reserve</t>
         </is>
@@ -3604,7 +3776,7 @@
         <f>IFERROR(O29/F29,"")</f>
         <v/>
       </c>
-      <c r="Q29" s="17" t="inlineStr">
+      <c r="Q29" s="36" t="inlineStr">
         <is>
           <t>Vendu</t>
         </is>
@@ -3701,7 +3873,7 @@
         <f>IFERROR(O30/F30,"")</f>
         <v/>
       </c>
-      <c r="Q30" s="14" t="inlineStr">
+      <c r="Q30" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -3798,7 +3970,7 @@
         <f>IFERROR(O31/F31,"")</f>
         <v/>
       </c>
-      <c r="Q31" s="16" t="inlineStr">
+      <c r="Q31" s="35" t="inlineStr">
         <is>
           <t>Optionne</t>
         </is>
@@ -3899,7 +4071,7 @@
         <f>IFERROR(O32/F32,"")</f>
         <v/>
       </c>
-      <c r="Q32" s="14" t="inlineStr">
+      <c r="Q32" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -3996,7 +4168,7 @@
         <f>IFERROR(O33/F33,"")</f>
         <v/>
       </c>
-      <c r="Q33" s="14" t="inlineStr">
+      <c r="Q33" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -4093,7 +4265,7 @@
         <f>IFERROR(O34/F34,"")</f>
         <v/>
       </c>
-      <c r="Q34" s="14" t="inlineStr">
+      <c r="Q34" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -4190,7 +4362,7 @@
         <f>IFERROR(O35/F35,"")</f>
         <v/>
       </c>
-      <c r="Q35" s="17" t="inlineStr">
+      <c r="Q35" s="36" t="inlineStr">
         <is>
           <t>Vendu</t>
         </is>
@@ -4287,7 +4459,7 @@
         <f>IFERROR(O36/F36,"")</f>
         <v/>
       </c>
-      <c r="Q36" s="14" t="inlineStr">
+      <c r="Q36" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -4384,7 +4556,7 @@
         <f>IFERROR(O37/F37,"")</f>
         <v/>
       </c>
-      <c r="Q37" s="14" t="inlineStr">
+      <c r="Q37" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -4477,7 +4649,7 @@
         <f>IFERROR(O38/F38,"")</f>
         <v/>
       </c>
-      <c r="Q38" s="14" t="inlineStr">
+      <c r="Q38" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -4570,7 +4742,7 @@
         <f>IFERROR(O39/F39,"")</f>
         <v/>
       </c>
-      <c r="Q39" s="16" t="inlineStr">
+      <c r="Q39" s="35" t="inlineStr">
         <is>
           <t>Optionne</t>
         </is>
@@ -4667,7 +4839,7 @@
         <f>IFERROR(O40/F40,"")</f>
         <v/>
       </c>
-      <c r="Q40" s="14" t="inlineStr">
+      <c r="Q40" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -4760,7 +4932,7 @@
         <f>IFERROR(O41/F41,"")</f>
         <v/>
       </c>
-      <c r="Q41" s="18" t="inlineStr">
+      <c r="Q41" s="37" t="inlineStr">
         <is>
           <t>Reserve</t>
         </is>
@@ -4853,7 +5025,7 @@
         <f>IFERROR(O42/F42,"")</f>
         <v/>
       </c>
-      <c r="Q42" s="14" t="inlineStr">
+      <c r="Q42" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -4950,7 +5122,7 @@
         <f>IFERROR(O43/F43,"")</f>
         <v/>
       </c>
-      <c r="Q43" s="14" t="inlineStr">
+      <c r="Q43" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -5047,7 +5219,7 @@
         <f>IFERROR(O44/F44,"")</f>
         <v/>
       </c>
-      <c r="Q44" s="14" t="inlineStr">
+      <c r="Q44" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -5140,7 +5312,7 @@
         <f>IFERROR(O45/F45,"")</f>
         <v/>
       </c>
-      <c r="Q45" s="14" t="inlineStr">
+      <c r="Q45" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -5233,7 +5405,7 @@
         <f>IFERROR(O46/F46,"")</f>
         <v/>
       </c>
-      <c r="Q46" s="19" t="inlineStr">
+      <c r="Q46" s="38" t="inlineStr">
         <is>
           <t>Bloque</t>
         </is>
@@ -5330,7 +5502,7 @@
         <f>IFERROR(O47/F47,"")</f>
         <v/>
       </c>
-      <c r="Q47" s="14" t="inlineStr">
+      <c r="Q47" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -5423,7 +5595,7 @@
         <f>IFERROR(O48/F48,"")</f>
         <v/>
       </c>
-      <c r="Q48" s="14" t="inlineStr">
+      <c r="Q48" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -5520,7 +5692,7 @@
         <f>IFERROR(O49/F49,"")</f>
         <v/>
       </c>
-      <c r="Q49" s="14" t="inlineStr">
+      <c r="Q49" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -5617,7 +5789,7 @@
         <f>IFERROR(O50/F50,"")</f>
         <v/>
       </c>
-      <c r="Q50" s="14" t="inlineStr">
+      <c r="Q50" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -5710,7 +5882,7 @@
         <f>IFERROR(O51/F51,"")</f>
         <v/>
       </c>
-      <c r="Q51" s="14" t="inlineStr">
+      <c r="Q51" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -5803,7 +5975,7 @@
         <f>IFERROR(O52/F52,"")</f>
         <v/>
       </c>
-      <c r="Q52" s="16" t="inlineStr">
+      <c r="Q52" s="35" t="inlineStr">
         <is>
           <t>Optionne</t>
         </is>
@@ -5900,7 +6072,7 @@
         <f>IFERROR(O53/F53,"")</f>
         <v/>
       </c>
-      <c r="Q53" s="17" t="inlineStr">
+      <c r="Q53" s="36" t="inlineStr">
         <is>
           <t>Vendu</t>
         </is>
@@ -5993,7 +6165,7 @@
         <f>IFERROR(O54/F54,"")</f>
         <v/>
       </c>
-      <c r="Q54" s="17" t="inlineStr">
+      <c r="Q54" s="36" t="inlineStr">
         <is>
           <t>Vendu</t>
         </is>
@@ -6090,7 +6262,7 @@
         <f>IFERROR(O55/F55,"")</f>
         <v/>
       </c>
-      <c r="Q55" s="14" t="inlineStr">
+      <c r="Q55" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -6187,7 +6359,7 @@
         <f>IFERROR(O56/F56,"")</f>
         <v/>
       </c>
-      <c r="Q56" s="14" t="inlineStr">
+      <c r="Q56" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -6284,7 +6456,7 @@
         <f>IFERROR(O57/F57,"")</f>
         <v/>
       </c>
-      <c r="Q57" s="14" t="inlineStr">
+      <c r="Q57" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -6381,7 +6553,7 @@
         <f>IFERROR(O58/F58,"")</f>
         <v/>
       </c>
-      <c r="Q58" s="16" t="inlineStr">
+      <c r="Q58" s="35" t="inlineStr">
         <is>
           <t>Optionne</t>
         </is>
@@ -6482,7 +6654,7 @@
         <f>IFERROR(O59/F59,"")</f>
         <v/>
       </c>
-      <c r="Q59" s="14" t="inlineStr">
+      <c r="Q59" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -6579,7 +6751,7 @@
         <f>IFERROR(O60/F60,"")</f>
         <v/>
       </c>
-      <c r="Q60" s="14" t="inlineStr">
+      <c r="Q60" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -6676,7 +6848,7 @@
         <f>IFERROR(O61/F61,"")</f>
         <v/>
       </c>
-      <c r="Q61" s="14" t="inlineStr">
+      <c r="Q61" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -6773,7 +6945,7 @@
         <f>IFERROR(O62/F62,"")</f>
         <v/>
       </c>
-      <c r="Q62" s="14" t="inlineStr">
+      <c r="Q62" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -6870,7 +7042,7 @@
         <f>IFERROR(O63/F63,"")</f>
         <v/>
       </c>
-      <c r="Q63" s="14" t="inlineStr">
+      <c r="Q63" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -6967,7 +7139,7 @@
         <f>IFERROR(O64/F64,"")</f>
         <v/>
       </c>
-      <c r="Q64" s="14" t="inlineStr">
+      <c r="Q64" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -7064,7 +7236,7 @@
         <f>IFERROR(O65/F65,"")</f>
         <v/>
       </c>
-      <c r="Q65" s="14" t="inlineStr">
+      <c r="Q65" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -7161,7 +7333,7 @@
         <f>IFERROR(O66/F66,"")</f>
         <v/>
       </c>
-      <c r="Q66" s="16" t="inlineStr">
+      <c r="Q66" s="35" t="inlineStr">
         <is>
           <t>Optionne</t>
         </is>
@@ -7262,7 +7434,7 @@
         <f>IFERROR(O67/F67,"")</f>
         <v/>
       </c>
-      <c r="Q67" s="14" t="inlineStr">
+      <c r="Q67" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -7355,7 +7527,7 @@
         <f>IFERROR(O68/F68,"")</f>
         <v/>
       </c>
-      <c r="Q68" s="14" t="inlineStr">
+      <c r="Q68" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -7448,7 +7620,7 @@
         <f>IFERROR(O69/F69,"")</f>
         <v/>
       </c>
-      <c r="Q69" s="14" t="inlineStr">
+      <c r="Q69" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -7541,7 +7713,7 @@
         <f>IFERROR(O70/F70,"")</f>
         <v/>
       </c>
-      <c r="Q70" s="14" t="inlineStr">
+      <c r="Q70" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -7634,7 +7806,7 @@
         <f>IFERROR(O71/F71,"")</f>
         <v/>
       </c>
-      <c r="Q71" s="14" t="inlineStr">
+      <c r="Q71" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -7727,7 +7899,7 @@
         <f>IFERROR(O72/F72,"")</f>
         <v/>
       </c>
-      <c r="Q72" s="17" t="inlineStr">
+      <c r="Q72" s="36" t="inlineStr">
         <is>
           <t>Vendu</t>
         </is>
@@ -7824,7 +7996,7 @@
         <f>IFERROR(O73/F73,"")</f>
         <v/>
       </c>
-      <c r="Q73" s="14" t="inlineStr">
+      <c r="Q73" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -7921,7 +8093,7 @@
         <f>IFERROR(O74/F74,"")</f>
         <v/>
       </c>
-      <c r="Q74" s="14" t="inlineStr">
+      <c r="Q74" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -8014,7 +8186,7 @@
         <f>IFERROR(O75/F75,"")</f>
         <v/>
       </c>
-      <c r="Q75" s="14" t="inlineStr">
+      <c r="Q75" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -8107,7 +8279,7 @@
         <f>IFERROR(O76/F76,"")</f>
         <v/>
       </c>
-      <c r="Q76" s="19" t="inlineStr">
+      <c r="Q76" s="38" t="inlineStr">
         <is>
           <t>Bloque</t>
         </is>
@@ -8204,7 +8376,7 @@
         <f>IFERROR(O77/F77,"")</f>
         <v/>
       </c>
-      <c r="Q77" s="14" t="inlineStr">
+      <c r="Q77" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -8297,7 +8469,7 @@
         <f>IFERROR(O78/F78,"")</f>
         <v/>
       </c>
-      <c r="Q78" s="14" t="inlineStr">
+      <c r="Q78" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -8394,7 +8566,7 @@
         <f>IFERROR(O79/F79,"")</f>
         <v/>
       </c>
-      <c r="Q79" s="14" t="inlineStr">
+      <c r="Q79" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -8491,7 +8663,7 @@
         <f>IFERROR(O80/F80,"")</f>
         <v/>
       </c>
-      <c r="Q80" s="14" t="inlineStr">
+      <c r="Q80" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -8584,7 +8756,7 @@
         <f>IFERROR(O81/F81,"")</f>
         <v/>
       </c>
-      <c r="Q81" s="14" t="inlineStr">
+      <c r="Q81" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -8677,7 +8849,7 @@
         <f>IFERROR(O82/F82,"")</f>
         <v/>
       </c>
-      <c r="Q82" s="14" t="inlineStr">
+      <c r="Q82" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -8770,7 +8942,7 @@
         <f>IFERROR(O83/F83,"")</f>
         <v/>
       </c>
-      <c r="Q83" s="14" t="inlineStr">
+      <c r="Q83" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -8863,7 +9035,7 @@
         <f>IFERROR(O84/F84,"")</f>
         <v/>
       </c>
-      <c r="Q84" s="14" t="inlineStr">
+      <c r="Q84" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -8960,7 +9132,7 @@
         <f>IFERROR(O85/F85,"")</f>
         <v/>
       </c>
-      <c r="Q85" s="14" t="inlineStr">
+      <c r="Q85" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -9057,7 +9229,7 @@
         <f>IFERROR(O86/F86,"")</f>
         <v/>
       </c>
-      <c r="Q86" s="14" t="inlineStr">
+      <c r="Q86" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -9154,7 +9326,7 @@
         <f>IFERROR(O87/F87,"")</f>
         <v/>
       </c>
-      <c r="Q87" s="14" t="inlineStr">
+      <c r="Q87" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -9251,7 +9423,7 @@
         <f>IFERROR(O88/F88,"")</f>
         <v/>
       </c>
-      <c r="Q88" s="14" t="inlineStr">
+      <c r="Q88" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -9348,7 +9520,7 @@
         <f>IFERROR(O89/F89,"")</f>
         <v/>
       </c>
-      <c r="Q89" s="18" t="inlineStr">
+      <c r="Q89" s="37" t="inlineStr">
         <is>
           <t>Reserve</t>
         </is>
@@ -9445,7 +9617,7 @@
         <f>IFERROR(O90/F90,"")</f>
         <v/>
       </c>
-      <c r="Q90" s="14" t="inlineStr">
+      <c r="Q90" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -9542,7 +9714,7 @@
         <f>IFERROR(O91/F91,"")</f>
         <v/>
       </c>
-      <c r="Q91" s="14" t="inlineStr">
+      <c r="Q91" s="34" t="inlineStr">
         <is>
           <t>Disponible</t>
         </is>
@@ -9572,6 +9744,23 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:W91"/>
+  <conditionalFormatting sqref="Q2:Q1000">
+    <cfRule type="containsText" priority="1" operator="containsText" dxfId="0" stopIfTrue="0" text="Disponible">
+      <formula>NOT(ISERROR(SEARCH("Disponible",Q2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="2" operator="containsText" dxfId="1" stopIfTrue="0" text="Optionne">
+      <formula>NOT(ISERROR(SEARCH("Optionne",Q2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="3" operator="containsText" dxfId="2" stopIfTrue="0" text="Reserve">
+      <formula>NOT(ISERROR(SEARCH("Reserve",Q2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="4" operator="containsText" dxfId="3" stopIfTrue="0" text="Vendu">
+      <formula>NOT(ISERROR(SEARCH("Vendu",Q2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" priority="5" operator="containsText" dxfId="4" stopIfTrue="0" text="Bloque">
+      <formula>NOT(ISERROR(SEARCH("Bloque",Q2)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="8">
     <dataValidation sqref="E2:E490" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Saisie invalide" error="Valeur non autorisee. Choisir dans la liste." type="list">
       <formula1>"Studio,F2,F3,F4,F5,Duplex,Bureau,Commerce"</formula1>
@@ -9634,6 +9823,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
@@ -9680,23 +9870,23 @@
           <t>A</t>
         </is>
       </c>
-      <c r="B6" s="24">
+      <c r="B6" s="39">
         <f>COUNTIFS(Lots!$B$2:$B$91,"A",Lots!$Q$2:$Q$91,"Disponible")</f>
         <v/>
       </c>
-      <c r="C6" s="25">
+      <c r="C6" s="40">
         <f>COUNTIFS(Lots!$B$2:$B$91,"A",Lots!$Q$2:$Q$91,"Optionne")</f>
         <v/>
       </c>
-      <c r="D6" s="26">
+      <c r="D6" s="41">
         <f>COUNTIFS(Lots!$B$2:$B$91,"A",Lots!$Q$2:$Q$91,"Reserve")</f>
         <v/>
       </c>
-      <c r="E6" s="27">
+      <c r="E6" s="42">
         <f>COUNTIFS(Lots!$B$2:$B$91,"A",Lots!$Q$2:$Q$91,"Vendu")</f>
         <v/>
       </c>
-      <c r="F6" s="28">
+      <c r="F6" s="43">
         <f>COUNTIFS(Lots!$B$2:$B$91,"A",Lots!$Q$2:$Q$91,"Bloque")</f>
         <v/>
       </c>
@@ -9711,23 +9901,23 @@
           <t>B</t>
         </is>
       </c>
-      <c r="B7" s="24">
+      <c r="B7" s="39">
         <f>COUNTIFS(Lots!$B$2:$B$91,"B",Lots!$Q$2:$Q$91,"Disponible")</f>
         <v/>
       </c>
-      <c r="C7" s="25">
+      <c r="C7" s="40">
         <f>COUNTIFS(Lots!$B$2:$B$91,"B",Lots!$Q$2:$Q$91,"Optionne")</f>
         <v/>
       </c>
-      <c r="D7" s="26">
+      <c r="D7" s="41">
         <f>COUNTIFS(Lots!$B$2:$B$91,"B",Lots!$Q$2:$Q$91,"Reserve")</f>
         <v/>
       </c>
-      <c r="E7" s="27">
+      <c r="E7" s="42">
         <f>COUNTIFS(Lots!$B$2:$B$91,"B",Lots!$Q$2:$Q$91,"Vendu")</f>
         <v/>
       </c>
-      <c r="F7" s="28">
+      <c r="F7" s="43">
         <f>COUNTIFS(Lots!$B$2:$B$91,"B",Lots!$Q$2:$Q$91,"Bloque")</f>
         <v/>
       </c>
@@ -9742,23 +9932,23 @@
           <t>C</t>
         </is>
       </c>
-      <c r="B8" s="24">
+      <c r="B8" s="39">
         <f>COUNTIFS(Lots!$B$2:$B$91,"C",Lots!$Q$2:$Q$91,"Disponible")</f>
         <v/>
       </c>
-      <c r="C8" s="25">
+      <c r="C8" s="40">
         <f>COUNTIFS(Lots!$B$2:$B$91,"C",Lots!$Q$2:$Q$91,"Optionne")</f>
         <v/>
       </c>
-      <c r="D8" s="26">
+      <c r="D8" s="41">
         <f>COUNTIFS(Lots!$B$2:$B$91,"C",Lots!$Q$2:$Q$91,"Reserve")</f>
         <v/>
       </c>
-      <c r="E8" s="27">
+      <c r="E8" s="42">
         <f>COUNTIFS(Lots!$B$2:$B$91,"C",Lots!$Q$2:$Q$91,"Vendu")</f>
         <v/>
       </c>
-      <c r="F8" s="28">
+      <c r="F8" s="43">
         <f>COUNTIFS(Lots!$B$2:$B$91,"C",Lots!$Q$2:$Q$91,"Bloque")</f>
         <v/>
       </c>
@@ -9767,6 +9957,7 @@
         <v/>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -9813,23 +10004,23 @@
           <t>Studio</t>
         </is>
       </c>
-      <c r="B12" s="24">
+      <c r="B12" s="39">
         <f>COUNTIFS(Lots!$E$2:$E$91,"Studio",Lots!$Q$2:$Q$91,"Disponible")</f>
         <v/>
       </c>
-      <c r="C12" s="25">
+      <c r="C12" s="40">
         <f>COUNTIFS(Lots!$E$2:$E$91,"Studio",Lots!$Q$2:$Q$91,"Optionne")</f>
         <v/>
       </c>
-      <c r="D12" s="26">
+      <c r="D12" s="41">
         <f>COUNTIFS(Lots!$E$2:$E$91,"Studio",Lots!$Q$2:$Q$91,"Reserve")</f>
         <v/>
       </c>
-      <c r="E12" s="27">
+      <c r="E12" s="42">
         <f>COUNTIFS(Lots!$E$2:$E$91,"Studio",Lots!$Q$2:$Q$91,"Vendu")</f>
         <v/>
       </c>
-      <c r="F12" s="28">
+      <c r="F12" s="43">
         <f>COUNTIFS(Lots!$E$2:$E$91,"Studio",Lots!$Q$2:$Q$91,"Bloque")</f>
         <v/>
       </c>
@@ -9844,23 +10035,23 @@
           <t>F2</t>
         </is>
       </c>
-      <c r="B13" s="24">
+      <c r="B13" s="39">
         <f>COUNTIFS(Lots!$E$2:$E$91,"F2",Lots!$Q$2:$Q$91,"Disponible")</f>
         <v/>
       </c>
-      <c r="C13" s="25">
+      <c r="C13" s="40">
         <f>COUNTIFS(Lots!$E$2:$E$91,"F2",Lots!$Q$2:$Q$91,"Optionne")</f>
         <v/>
       </c>
-      <c r="D13" s="26">
+      <c r="D13" s="41">
         <f>COUNTIFS(Lots!$E$2:$E$91,"F2",Lots!$Q$2:$Q$91,"Reserve")</f>
         <v/>
       </c>
-      <c r="E13" s="27">
+      <c r="E13" s="42">
         <f>COUNTIFS(Lots!$E$2:$E$91,"F2",Lots!$Q$2:$Q$91,"Vendu")</f>
         <v/>
       </c>
-      <c r="F13" s="28">
+      <c r="F13" s="43">
         <f>COUNTIFS(Lots!$E$2:$E$91,"F2",Lots!$Q$2:$Q$91,"Bloque")</f>
         <v/>
       </c>
@@ -9875,23 +10066,23 @@
           <t>F3</t>
         </is>
       </c>
-      <c r="B14" s="24">
+      <c r="B14" s="39">
         <f>COUNTIFS(Lots!$E$2:$E$91,"F3",Lots!$Q$2:$Q$91,"Disponible")</f>
         <v/>
       </c>
-      <c r="C14" s="25">
+      <c r="C14" s="40">
         <f>COUNTIFS(Lots!$E$2:$E$91,"F3",Lots!$Q$2:$Q$91,"Optionne")</f>
         <v/>
       </c>
-      <c r="D14" s="26">
+      <c r="D14" s="41">
         <f>COUNTIFS(Lots!$E$2:$E$91,"F3",Lots!$Q$2:$Q$91,"Reserve")</f>
         <v/>
       </c>
-      <c r="E14" s="27">
+      <c r="E14" s="42">
         <f>COUNTIFS(Lots!$E$2:$E$91,"F3",Lots!$Q$2:$Q$91,"Vendu")</f>
         <v/>
       </c>
-      <c r="F14" s="28">
+      <c r="F14" s="43">
         <f>COUNTIFS(Lots!$E$2:$E$91,"F3",Lots!$Q$2:$Q$91,"Bloque")</f>
         <v/>
       </c>
@@ -9906,23 +10097,23 @@
           <t>F4</t>
         </is>
       </c>
-      <c r="B15" s="24">
+      <c r="B15" s="39">
         <f>COUNTIFS(Lots!$E$2:$E$91,"F4",Lots!$Q$2:$Q$91,"Disponible")</f>
         <v/>
       </c>
-      <c r="C15" s="25">
+      <c r="C15" s="40">
         <f>COUNTIFS(Lots!$E$2:$E$91,"F4",Lots!$Q$2:$Q$91,"Optionne")</f>
         <v/>
       </c>
-      <c r="D15" s="26">
+      <c r="D15" s="41">
         <f>COUNTIFS(Lots!$E$2:$E$91,"F4",Lots!$Q$2:$Q$91,"Reserve")</f>
         <v/>
       </c>
-      <c r="E15" s="27">
+      <c r="E15" s="42">
         <f>COUNTIFS(Lots!$E$2:$E$91,"F4",Lots!$Q$2:$Q$91,"Vendu")</f>
         <v/>
       </c>
-      <c r="F15" s="28">
+      <c r="F15" s="43">
         <f>COUNTIFS(Lots!$E$2:$E$91,"F4",Lots!$Q$2:$Q$91,"Bloque")</f>
         <v/>
       </c>
@@ -9937,23 +10128,23 @@
           <t>Duplex</t>
         </is>
       </c>
-      <c r="B16" s="24">
+      <c r="B16" s="39">
         <f>COUNTIFS(Lots!$E$2:$E$91,"Duplex",Lots!$Q$2:$Q$91,"Disponible")</f>
         <v/>
       </c>
-      <c r="C16" s="25">
+      <c r="C16" s="40">
         <f>COUNTIFS(Lots!$E$2:$E$91,"Duplex",Lots!$Q$2:$Q$91,"Optionne")</f>
         <v/>
       </c>
-      <c r="D16" s="26">
+      <c r="D16" s="41">
         <f>COUNTIFS(Lots!$E$2:$E$91,"Duplex",Lots!$Q$2:$Q$91,"Reserve")</f>
         <v/>
       </c>
-      <c r="E16" s="27">
+      <c r="E16" s="42">
         <f>COUNTIFS(Lots!$E$2:$E$91,"Duplex",Lots!$Q$2:$Q$91,"Vendu")</f>
         <v/>
       </c>
-      <c r="F16" s="28">
+      <c r="F16" s="43">
         <f>COUNTIFS(Lots!$E$2:$E$91,"Duplex",Lots!$Q$2:$Q$91,"Bloque")</f>
         <v/>
       </c>
@@ -9968,23 +10159,23 @@
           <t>Bureau</t>
         </is>
       </c>
-      <c r="B17" s="24">
+      <c r="B17" s="39">
         <f>COUNTIFS(Lots!$E$2:$E$91,"Bureau",Lots!$Q$2:$Q$91,"Disponible")</f>
         <v/>
       </c>
-      <c r="C17" s="25">
+      <c r="C17" s="40">
         <f>COUNTIFS(Lots!$E$2:$E$91,"Bureau",Lots!$Q$2:$Q$91,"Optionne")</f>
         <v/>
       </c>
-      <c r="D17" s="26">
+      <c r="D17" s="41">
         <f>COUNTIFS(Lots!$E$2:$E$91,"Bureau",Lots!$Q$2:$Q$91,"Reserve")</f>
         <v/>
       </c>
-      <c r="E17" s="27">
+      <c r="E17" s="42">
         <f>COUNTIFS(Lots!$E$2:$E$91,"Bureau",Lots!$Q$2:$Q$91,"Vendu")</f>
         <v/>
       </c>
-      <c r="F17" s="28">
+      <c r="F17" s="43">
         <f>COUNTIFS(Lots!$E$2:$E$91,"Bureau",Lots!$Q$2:$Q$91,"Bloque")</f>
         <v/>
       </c>
@@ -9999,23 +10190,23 @@
           <t>Commerce</t>
         </is>
       </c>
-      <c r="B18" s="24">
+      <c r="B18" s="39">
         <f>COUNTIFS(Lots!$E$2:$E$91,"Commerce",Lots!$Q$2:$Q$91,"Disponible")</f>
         <v/>
       </c>
-      <c r="C18" s="25">
+      <c r="C18" s="40">
         <f>COUNTIFS(Lots!$E$2:$E$91,"Commerce",Lots!$Q$2:$Q$91,"Optionne")</f>
         <v/>
       </c>
-      <c r="D18" s="26">
+      <c r="D18" s="41">
         <f>COUNTIFS(Lots!$E$2:$E$91,"Commerce",Lots!$Q$2:$Q$91,"Reserve")</f>
         <v/>
       </c>
-      <c r="E18" s="27">
+      <c r="E18" s="42">
         <f>COUNTIFS(Lots!$E$2:$E$91,"Commerce",Lots!$Q$2:$Q$91,"Vendu")</f>
         <v/>
       </c>
-      <c r="F18" s="28">
+      <c r="F18" s="43">
         <f>COUNTIFS(Lots!$E$2:$E$91,"Commerce",Lots!$Q$2:$Q$91,"Bloque")</f>
         <v/>
       </c>
@@ -10024,6 +10215,7 @@
         <v/>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
@@ -10070,23 +10262,23 @@
           <t>Rue</t>
         </is>
       </c>
-      <c r="B22" s="24">
+      <c r="B22" s="39">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Rue",Lots!$Q$2:$Q$91,"Disponible")</f>
         <v/>
       </c>
-      <c r="C22" s="25">
+      <c r="C22" s="40">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Rue",Lots!$Q$2:$Q$91,"Optionne")</f>
         <v/>
       </c>
-      <c r="D22" s="26">
+      <c r="D22" s="41">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Rue",Lots!$Q$2:$Q$91,"Reserve")</f>
         <v/>
       </c>
-      <c r="E22" s="27">
+      <c r="E22" s="42">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Rue",Lots!$Q$2:$Q$91,"Vendu")</f>
         <v/>
       </c>
-      <c r="F22" s="28">
+      <c r="F22" s="43">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Rue",Lots!$Q$2:$Q$91,"Bloque")</f>
         <v/>
       </c>
@@ -10101,23 +10293,23 @@
           <t>Cour</t>
         </is>
       </c>
-      <c r="B23" s="24">
+      <c r="B23" s="39">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Cour",Lots!$Q$2:$Q$91,"Disponible")</f>
         <v/>
       </c>
-      <c r="C23" s="25">
+      <c r="C23" s="40">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Cour",Lots!$Q$2:$Q$91,"Optionne")</f>
         <v/>
       </c>
-      <c r="D23" s="26">
+      <c r="D23" s="41">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Cour",Lots!$Q$2:$Q$91,"Reserve")</f>
         <v/>
       </c>
-      <c r="E23" s="27">
+      <c r="E23" s="42">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Cour",Lots!$Q$2:$Q$91,"Vendu")</f>
         <v/>
       </c>
-      <c r="F23" s="28">
+      <c r="F23" s="43">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Cour",Lots!$Q$2:$Q$91,"Bloque")</f>
         <v/>
       </c>
@@ -10132,23 +10324,23 @@
           <t>Jardin</t>
         </is>
       </c>
-      <c r="B24" s="24">
+      <c r="B24" s="39">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Jardin",Lots!$Q$2:$Q$91,"Disponible")</f>
         <v/>
       </c>
-      <c r="C24" s="25">
+      <c r="C24" s="40">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Jardin",Lots!$Q$2:$Q$91,"Optionne")</f>
         <v/>
       </c>
-      <c r="D24" s="26">
+      <c r="D24" s="41">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Jardin",Lots!$Q$2:$Q$91,"Reserve")</f>
         <v/>
       </c>
-      <c r="E24" s="27">
+      <c r="E24" s="42">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Jardin",Lots!$Q$2:$Q$91,"Vendu")</f>
         <v/>
       </c>
-      <c r="F24" s="28">
+      <c r="F24" s="43">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Jardin",Lots!$Q$2:$Q$91,"Bloque")</f>
         <v/>
       </c>
@@ -10163,23 +10355,23 @@
           <t>Double orientation</t>
         </is>
       </c>
-      <c r="B25" s="24">
+      <c r="B25" s="39">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Double orientation",Lots!$Q$2:$Q$91,"Disponible")</f>
         <v/>
       </c>
-      <c r="C25" s="25">
+      <c r="C25" s="40">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Double orientation",Lots!$Q$2:$Q$91,"Optionne")</f>
         <v/>
       </c>
-      <c r="D25" s="26">
+      <c r="D25" s="41">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Double orientation",Lots!$Q$2:$Q$91,"Reserve")</f>
         <v/>
       </c>
-      <c r="E25" s="27">
+      <c r="E25" s="42">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Double orientation",Lots!$Q$2:$Q$91,"Vendu")</f>
         <v/>
       </c>
-      <c r="F25" s="28">
+      <c r="F25" s="43">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Double orientation",Lots!$Q$2:$Q$91,"Bloque")</f>
         <v/>
       </c>
@@ -10194,23 +10386,23 @@
           <t>Angle</t>
         </is>
       </c>
-      <c r="B26" s="24">
+      <c r="B26" s="39">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Angle",Lots!$Q$2:$Q$91,"Disponible")</f>
         <v/>
       </c>
-      <c r="C26" s="25">
+      <c r="C26" s="40">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Angle",Lots!$Q$2:$Q$91,"Optionne")</f>
         <v/>
       </c>
-      <c r="D26" s="26">
+      <c r="D26" s="41">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Angle",Lots!$Q$2:$Q$91,"Reserve")</f>
         <v/>
       </c>
-      <c r="E26" s="27">
+      <c r="E26" s="42">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Angle",Lots!$Q$2:$Q$91,"Vendu")</f>
         <v/>
       </c>
-      <c r="F26" s="28">
+      <c r="F26" s="43">
         <f>COUNTIFS(Lots!$K$2:$K$91,"Angle",Lots!$Q$2:$Q$91,"Bloque")</f>
         <v/>
       </c>
@@ -10219,6 +10411,7 @@
         <v/>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>

</xml_diff>